<commit_message>
🛡️ Sentinel: Fix 5 more security vulnerabilities (Cookies, Session Encryption, Path Traversal, Error Leak, APP_KEY)
6. [HIGH] Insecure cookies — added HttpOnly, Secure, SameSite=Strict
7. [HIGH] Weak session encryption (base64) — replaced with AES-256-CBC
8. [HIGH] Path traversal in Session::make() — sanitize key with regex
9. [MEDIUM] Database error leak — log internally, show generic message
10. [MEDIUM] Missing APP_KEY — added to .env.example
</commit_message>
<xml_diff>
--- a/Security_Findings_Report.xlsx
+++ b/Security_Findings_Report.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Security Findings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="الملخص" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -460,13 +460,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="50" customWidth="1" min="7" max="7"/>
@@ -477,47 +477,47 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>#</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Severity</t>
+          <t>الخطورة</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Vulnerability</t>
+          <t>الثغرة</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>File</t>
+          <t>الملف</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Line</t>
+          <t>السطر</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>الوصف</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Impact</t>
+          <t>التأثير</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Fix Applied</t>
+          <t>الإصلاح</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>الحالة</t>
         </is>
       </c>
     </row>
@@ -527,12 +527,12 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>عالي</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>SQL Injection in signIn()</t>
+          <t>حقن SQL في دالة signIn()</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -547,22 +547,22 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>User-supplied keys in signIn() were used directly in SQL query without validation. An attacker could inject arbitrary SQL by crafting malicious array keys in the login request.</t>
+          <t>مفاتيح المقدمة من المستخدم كانت تُستخدم مباشرة في استعلام SQL بدون تحقق. يمكن للمهاجم حقن SQL عشوائي عبر إنشاء مفاتيح خبيثة.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Authentication bypass, data leakage, database manipulation</t>
+          <t>تجاوز المصادقة، تسريب البيانات، التلاعب بقاعدة البيانات</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Added whitelist validation against allowed column names from AuthParams.json. Only known column names are used in SQL queries.</t>
+          <t>أضفنا تحقق القائمة البيضاء مقابل أسماء الأعمدة المسموحة من AuthParams.json</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>FIXED</t>
+          <t>تم الإصلاح</t>
         </is>
       </c>
     </row>
@@ -572,12 +572,12 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>عالي</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Path Traversal in Router</t>
+          <t>تجاوز المسار في الراوتر</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -592,22 +592,22 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>The page parameter was used directly in file_exists() without sanitization. An attacker could use ../ sequences to traverse directories and access arbitrary files on the server.</t>
+          <t>معلمة الصفحة كانت تُستخدم مباشرة في file_exists() بدون تنقية. يمكن للمهاجم استخدام ../ لتجاوز المجلدات.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Arbitrary file read, source code disclosure, potential RCE</t>
+          <t>قراءة ملفات عشوائية، الكشف عن الكود المصدري، تنفيذ تعليمات برمجية</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Added regex validation to only allow alphanumeric characters, dashes, underscores, and slashes in the page parameter.</t>
+          <t>أضفنا تحقق regex للسماح بالأحرف والأرقام والشرطات فقط</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>FIXED</t>
+          <t>تم الإصلاح</t>
         </is>
       </c>
     </row>
@@ -617,12 +617,12 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>عالي</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>SSRF in Webhook</t>
+          <t>ثغرة SSRF في Webhook</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -637,22 +637,22 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>The webhook URL was not validated against internal/private IP ranges. An attacker could send requests to internal services (localhost, 169.254.169.254 for cloud metadata, private network services).</t>
+          <t>عنوان URL لم يكن يُتحقق منه مقابل نطاقات IP الداخلية/الخاصة. يمكن إرسال طلبات للخدمات الداخلية.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Internal service access, cloud metadata theft, port scanning, data exfiltration</t>
+          <t>الوصول للخدمات الداخلية، سرقة بيانات التعريف السحابية، فحص المنافذ</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Added HTTPS-only enforcement, DNS resolution to IP, and filtering of private/reserved IP ranges. Added connection timeout.</t>
+          <t>أضفنا فرض HTTPS، تحليل DNS، وتصفية نطاقات IP الخاصة</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>FIXED</t>
+          <t>تم الإصلاح</t>
         </is>
       </c>
     </row>
@@ -662,12 +662,12 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>متوسط</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Missing Security Headers</t>
+          <t>غياب رؤوس الأمان</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -677,27 +677,27 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>غير محدد</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>No security headers were configured. Missing X-Content-Type-Options, X-Frame-Options, X-XSS-Protection, Referrer-Policy, and Permissions-Policy headers.</t>
+          <t>لم تكن هناك رؤوس أمان مُكوّنة. مفقودة: X-Content-Type-Options, X-Frame-Options, X-XSS-Protection</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Clickjacking, MIME-type sniffing attacks, XSS amplification, referrer leakage</t>
+          <t>Clickjacking, MIME sniffing, XSS amplification, تسريب referrer</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Added comprehensive security headers in .htaccess: nosniff, SAMEORIGIN, XSS protection, strict referrer policy, and permissions policy.</t>
+          <t>أضفنا رؤوس أمان شاملة في .htaccess</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>FIXED</t>
+          <t>تم الإصلاح</t>
         </is>
       </c>
     </row>
@@ -707,12 +707,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>متوسط</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Session Fixation</t>
+          <t>تثبيت الجلسة</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -727,22 +727,247 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>After successful login, the session ID was not regenerated. An attacker could fixate a session ID and hijack the user after they authenticate.</t>
+          <t>لم يتم تجديد معرف الجلسة بعد تسجيل الدخول الناجح. يمكن للمهاجم تثبيت معرف الجلسة واختطافها.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Session hijacking, account takeover</t>
+          <t>اختطاف الجلسة، الاستيلاء على الحساب</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Added session_regenerate_id(true) after successful authentication to create a new session ID.</t>
+          <t>أضفنا session_regenerate_id(true) بعد المصادقة الناجحة</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>FIXED</t>
+          <t>تم الإصلاح</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>عالي</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>ملفات تعريف الارتباط غير الآمنة</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>core/functions/PHP/classes/CookieManager.php</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>ملفات تعريف الارتباط لم تكن تحتوي على علامات الأمان HttpOnly و Secure و SameSite.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>سرقة ملفات تعريف الارتباط عبر XSS, هجمات CSRF</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>أضفنا خيارات setcookie الآمنة: HttpOnly, Secure, SameSite=Strict</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>تم الإصلاح</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>عالي</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>تشفير الجلسات ضعيف (base64)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>core/functions/PHP/classes/Session.php</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>89</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>التشفير المستخدم كان base64 فقط وهو ليس تشفيراً حقيقياً. يمكن فك ترميز البيانات بسهولة.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>تسريب بيانات الجلسة الحساسة, cookies, بيانات الاعتماد</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>استبدلنا base64 بتشفير AES-256-CBC مع IV عشوائي</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>تم الإصلاح</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>عالي</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>تجاوز المسار في الجلسات</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>core/functions/PHP/classes/Session.php</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>مفتاح الجلسة لم يكن يُنقى، مما يسمح باستخدام ../ في أسماء المفاتيح لكتابة ملفات خارج مجلد الجلسات.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>كتابة ملفات عشوائية, تنفيذ تعليمات برمجية عن بُعد</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>أضفنا تنقية للمفتاح بـ regex للسماح بالأحرف والأرقام فقط</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>تم الإصلاح</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>متوسط</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>تسريب معلومات حساسة في رسائل الخطأ</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>core/functions/PHP/classes/Database.php</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>رسالة خطأ قاعدة البيانات كانت تكشف تفاصيل الخطأ للمستخدم.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>الكشف عن معلومات حساسة: مسارات الملفات, أسماء الجداول, بيانات الاعتماد</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>أضفنا error_log داخلي وإظهار رسالة خطأ عامة بدون تفاصيل</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>تم الإصلاح</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>متوسط</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>مفتاح تشفير APP_KEY مفقود</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>.env.example</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>غير محدد</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>لم يكن هناك متغير APP_KEY في ملف البيئة، مما يعني أن التشفير يستخدم مفتاح افتراضي ضعيف.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>فك تشفير البيانات الحساسة, التلاعب بالجلسات</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>أضفنا APP_KEY إلى .env.example مع توضيح ضرورة تغييره</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>تم الإصلاح</t>
         </is>
       </c>
     </row>
@@ -763,56 +988,56 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Security Scan Summary</t>
+          <t>ملخص فحص الأمان</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Scan Date: 2026-09-08</t>
+          <t>تاريخ الفحص: 2026-09-08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Total Findings: 5</t>
+          <t>إجمالي الثغرات: 10</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Critical: 0</t>
+          <t>حرج: 0</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>High: 3</t>
+          <t>عالي: 5</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Medium: 2</t>
+          <t>متوسط: 5</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Low: 0</t>
+          <t>منخفض: 0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>All Fixed: 5/5</t>
+          <t>تم الإصلاح: 10/10</t>
         </is>
       </c>
     </row>

</xml_diff>